<commit_message>
code updated final one
</commit_message>
<xml_diff>
--- a/shivshankar_agile_template.xlsx
+++ b/shivshankar_agile_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Downloads\infosys\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5E16823C-6F5A-433F-B794-4EB8F9EC3703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522919B2-BA8A-408A-88AD-E0AA4BA0084B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -4617,7 +4617,7 @@
         <v>10</v>
       </c>
       <c r="D5" s="14">
-        <v>45600</v>
+        <v>45631</v>
       </c>
       <c r="E5" s="14">
         <v>45602</v>
@@ -4688,7 +4688,7 @@
         <v>15</v>
       </c>
       <c r="D6" s="14">
-        <v>45603</v>
+        <v>45633</v>
       </c>
       <c r="E6" s="14">
         <v>45604</v>
@@ -4759,7 +4759,7 @@
         <v>20</v>
       </c>
       <c r="D7" s="14">
-        <v>45607</v>
+        <v>45637</v>
       </c>
       <c r="E7" s="14">
         <v>45607</v>
@@ -4830,7 +4830,7 @@
         <v>24</v>
       </c>
       <c r="D8" s="14">
-        <v>45608</v>
+        <v>45638</v>
       </c>
       <c r="E8" s="14">
         <v>45611</v>
@@ -4901,7 +4901,7 @@
         <v>28</v>
       </c>
       <c r="D9" s="14">
-        <v>45612</v>
+        <v>45642</v>
       </c>
       <c r="E9" s="14">
         <v>45618</v>
@@ -4972,7 +4972,7 @@
         <v>32</v>
       </c>
       <c r="D10" s="14">
-        <v>45619</v>
+        <v>45649</v>
       </c>
       <c r="E10" s="14">
         <v>45625</v>
@@ -5043,7 +5043,7 @@
         <v>36</v>
       </c>
       <c r="D11" s="14">
-        <v>45628</v>
+        <v>45659</v>
       </c>
       <c r="E11" s="14">
         <v>45632</v>
@@ -5114,7 +5114,7 @@
         <v>38</v>
       </c>
       <c r="D12" s="22">
-        <v>45635</v>
+        <v>45666</v>
       </c>
       <c r="E12" s="22">
         <v>45639</v>
@@ -5185,7 +5185,7 @@
         <v>42</v>
       </c>
       <c r="D13" s="14">
-        <v>45642</v>
+        <v>45674</v>
       </c>
       <c r="E13" s="14">
         <v>45646</v>
@@ -5256,7 +5256,7 @@
         <v>46</v>
       </c>
       <c r="D14" s="14">
-        <v>45649</v>
+        <v>45680</v>
       </c>
       <c r="E14" s="14">
         <v>45653</v>
@@ -7592,10 +7592,10 @@
         <v>88</v>
       </c>
       <c r="C2" s="38">
-        <v>45600</v>
+        <v>45631</v>
       </c>
       <c r="D2" s="38">
-        <v>45602</v>
+        <v>45326</v>
       </c>
       <c r="E2" s="15" t="s">
         <v>139</v>
@@ -7621,10 +7621,10 @@
         <v>98</v>
       </c>
       <c r="C3" s="38">
-        <v>45612</v>
+        <v>45642</v>
       </c>
       <c r="D3" s="38">
-        <v>45618</v>
+        <v>45648</v>
       </c>
       <c r="E3" s="15" t="s">
         <v>139</v>
@@ -7650,10 +7650,10 @@
         <v>101</v>
       </c>
       <c r="C4" s="38">
-        <v>45619</v>
+        <v>45649</v>
       </c>
       <c r="D4" s="38">
-        <v>45625</v>
+        <v>45655</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>139</v>
@@ -7679,10 +7679,10 @@
         <v>134</v>
       </c>
       <c r="C5" s="38">
-        <v>45628</v>
+        <v>45656</v>
       </c>
       <c r="D5" s="38">
-        <v>45632</v>
+        <v>45672</v>
       </c>
       <c r="E5" s="15" t="s">
         <v>139</v>

</xml_diff>